<commit_message>
Se agrega referencia sobre factor de escala y se documenta, se documentan los valores de referencia de XFLR5 y se procesan para obtener el momento de bisagra y su relación con el ángulo de ataque. Se agregan los archivos de resultados de XFLR5 para Mach 0.4, 0.5 y 0.6 a 0 msnm. Se descubre que el factor de escala de 0.25 era muy bajo y se proponen unos nuevos tentativos.
</commit_message>
<xml_diff>
--- a/04_CFD/00_XFLR5/Nalci&Kayran/Mach 0_4 0 msnm.xlsx
+++ b/04_CFD/00_XFLR5/Nalci&Kayran/Mach 0_4 0 msnm.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udeconce-my.sharepoint.com/personal/joarriagada2021_udec_cl/Documents/Escritorio/Memoria/04_CFD/00_XFLR5/Nalci&amp;Kayran/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{BE7D5C80-A819-4064-BA83-A94058516697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{117372FB-40BD-4814-A20A-2D21C7528795}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{BE7D5C80-A819-4064-BA83-A94058516697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F58663FD-676C-40F0-9902-95F65AE572F1}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{FE690B17-51F1-4F28-8DB9-6B77EB255480}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{FE690B17-51F1-4F28-8DB9-6B77EB255480}"/>
   </bookViews>
   <sheets>
     <sheet name="Mach 0_4 0 msnm" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1087,8 +1100,8 @@
         <v>11345.466125000001</v>
       </c>
       <c r="O8">
-        <f>I8*N8*0.18*0.121333</f>
-        <v>-19.366077491490937</v>
+        <f>I8*N8*0.018*0.121333</f>
+        <v>-1.9366077491490936</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1136,8 +1149,8 @@
         <v>11345.466125000001</v>
       </c>
       <c r="O9">
-        <f t="shared" ref="O9:O72" si="1">I9*N9*0.18*0.121333</f>
-        <v>-19.072453096652126</v>
+        <f t="shared" ref="O9:O72" si="1">I9*N9*0.018*0.121333</f>
+        <v>-1.9072453096652124</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1186,7 +1199,7 @@
       </c>
       <c r="O10">
         <f t="shared" si="1"/>
-        <v>-18.77709421171722</v>
+        <v>-1.8777094211717222</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -1235,7 +1248,7 @@
       </c>
       <c r="O11">
         <f t="shared" si="1"/>
-        <v>-18.480496405285109</v>
+        <v>-1.848049640528511</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -1284,7 +1297,7 @@
       </c>
       <c r="O12">
         <f t="shared" si="1"/>
-        <v>-18.182411893056344</v>
+        <v>-1.8182411893056343</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1333,7 +1346,7 @@
       </c>
       <c r="O13">
         <f t="shared" si="1"/>
-        <v>-17.88308845933037</v>
+        <v>-1.788308845933037</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1382,7 +1395,7 @@
       </c>
       <c r="O14">
         <f t="shared" si="1"/>
-        <v>-17.582278319807738</v>
+        <v>-1.7582278319807738</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1431,7 +1444,7 @@
       </c>
       <c r="O15">
         <f t="shared" si="1"/>
-        <v>-17.280229258787902</v>
+        <v>-1.7280229258787903</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1480,7 +1493,7 @@
       </c>
       <c r="O16">
         <f t="shared" si="1"/>
-        <v>-16.976941276270857</v>
+        <v>-1.6976941276270858</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -1529,7 +1542,7 @@
       </c>
       <c r="O17">
         <f t="shared" si="1"/>
-        <v>-16.672166587957157</v>
+        <v>-1.6672166587957156</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -1578,7 +1591,7 @@
       </c>
       <c r="O18">
         <f t="shared" si="1"/>
-        <v>-16.366152978146246</v>
+        <v>-1.6366152978146244</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -1627,7 +1640,7 @@
       </c>
       <c r="O19">
         <f t="shared" si="1"/>
-        <v>-16.059148231137566</v>
+        <v>-1.6059148231137566</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
@@ -1676,7 +1689,7 @@
       </c>
       <c r="O20">
         <f t="shared" si="1"/>
-        <v>-15.750656778332235</v>
+        <v>-1.5750656778332235</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1725,7 +1738,7 @@
       </c>
       <c r="O21">
         <f t="shared" si="1"/>
-        <v>-15.441174188329141</v>
+        <v>-1.5441174188329139</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -1774,7 +1787,7 @@
       </c>
       <c r="O22">
         <f t="shared" si="1"/>
-        <v>-15.130452676828829</v>
+        <v>-1.5130452676828829</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -1823,7 +1836,7 @@
       </c>
       <c r="O23">
         <f t="shared" si="1"/>
-        <v>-14.818492243831313</v>
+        <v>-1.4818492243831312</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -1872,7 +1885,7 @@
       </c>
       <c r="O24">
         <f t="shared" si="1"/>
-        <v>-14.505540673636025</v>
+        <v>-1.4505540673636024</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -1921,7 +1934,7 @@
       </c>
       <c r="O25">
         <f t="shared" si="1"/>
-        <v>-14.191350181943527</v>
+        <v>-1.4191350181943525</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -1970,7 +1983,7 @@
       </c>
       <c r="O26">
         <f t="shared" si="1"/>
-        <v>-13.876168553053263</v>
+        <v>-1.3876168553053263</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -2019,7 +2032,7 @@
       </c>
       <c r="O27">
         <f t="shared" si="1"/>
-        <v>-13.559995786965231</v>
+        <v>-1.3559995786965229</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -2068,7 +2081,7 @@
       </c>
       <c r="O28">
         <f t="shared" si="1"/>
-        <v>-13.242831883679429</v>
+        <v>-1.3242831883679427</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -2117,7 +2130,7 @@
       </c>
       <c r="O29">
         <f t="shared" si="1"/>
-        <v>-12.924676843195858</v>
+        <v>-1.2924676843195855</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -2166,7 +2179,7 @@
       </c>
       <c r="O30">
         <f t="shared" si="1"/>
-        <v>-12.605282881215077</v>
+        <v>-1.2605282881215076</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -2215,7 +2228,7 @@
       </c>
       <c r="O31">
         <f t="shared" si="1"/>
-        <v>-12.28514556633597</v>
+        <v>-1.2285145566335971</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -2264,7 +2277,7 @@
       </c>
       <c r="O32">
         <f t="shared" si="1"/>
-        <v>-11.96426489855854</v>
+        <v>-1.1964264898558539</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -2313,7 +2326,7 @@
       </c>
       <c r="O33">
         <f t="shared" si="1"/>
-        <v>-11.642145309283897</v>
+        <v>-1.1642145309283896</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
@@ -2362,7 +2375,7 @@
       </c>
       <c r="O34">
         <f t="shared" si="1"/>
-        <v>-11.319282367110929</v>
+        <v>-1.131928236711093</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
@@ -2411,7 +2424,7 @@
       </c>
       <c r="O35">
         <f t="shared" si="1"/>
-        <v>-10.995676072039634</v>
+        <v>-1.0995676072039635</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
@@ -2460,7 +2473,7 @@
       </c>
       <c r="O36">
         <f t="shared" si="1"/>
-        <v>-10.671078639770572</v>
+        <v>-1.067107863977057</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
@@ -2509,7 +2522,7 @@
       </c>
       <c r="O37">
         <f t="shared" si="1"/>
-        <v>-10.345737854603183</v>
+        <v>-1.0345737854603183</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
@@ -2558,7 +2571,7 @@
       </c>
       <c r="O38">
         <f t="shared" si="1"/>
-        <v>-10.019653716537469</v>
+        <v>-1.0019653716537467</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
@@ -2607,7 +2620,7 @@
       </c>
       <c r="O39">
         <f t="shared" si="1"/>
-        <v>-9.6928262255734268</v>
+        <v>-0.96928262255734277</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
@@ -2656,7 +2669,7 @@
       </c>
       <c r="O40">
         <f t="shared" si="1"/>
-        <v>-9.3652553817110604</v>
+        <v>-0.93652553817110618</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
@@ -2705,7 +2718,7 @@
       </c>
       <c r="O41">
         <f t="shared" si="1"/>
-        <v>-9.0369411849503685</v>
+        <v>-0.90369411849503678</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
@@ -2754,7 +2767,7 @@
       </c>
       <c r="O42">
         <f t="shared" si="1"/>
-        <v>-8.7078836352913491</v>
+        <v>-0.8707883635291348</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
@@ -2803,7 +2816,7 @@
       </c>
       <c r="O43">
         <f t="shared" si="1"/>
-        <v>-8.3783305170334454</v>
+        <v>-0.83783305170334454</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
@@ -2852,7 +2865,7 @@
       </c>
       <c r="O44">
         <f t="shared" si="1"/>
-        <v>-8.0480340458772162</v>
+        <v>-0.80480340458772159</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
@@ -2901,7 +2914,7 @@
       </c>
       <c r="O45">
         <f t="shared" si="1"/>
-        <v>-7.7172420061221025</v>
+        <v>-0.77172420061221014</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
@@ -2950,7 +2963,7 @@
       </c>
       <c r="O46">
         <f t="shared" si="1"/>
-        <v>-7.3859543977681055</v>
+        <v>-0.73859543977681041</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
@@ -2999,7 +3012,7 @@
       </c>
       <c r="O47">
         <f t="shared" si="1"/>
-        <v>-7.0539234365157819</v>
+        <v>-0.7053923436515781</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
@@ -3048,7 +3061,7 @@
       </c>
       <c r="O48">
         <f t="shared" si="1"/>
-        <v>-6.7213969066645731</v>
+        <v>-0.67213969066645729</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
@@ -3097,7 +3110,7 @@
       </c>
       <c r="O49">
         <f t="shared" si="1"/>
-        <v>-6.3883748082144827</v>
+        <v>-0.6388374808214482</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
@@ -3146,7 +3159,7 @@
       </c>
       <c r="O50">
         <f t="shared" si="1"/>
-        <v>-6.054857141165507</v>
+        <v>-0.60548571411655061</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
@@ -3195,7 +3208,7 @@
       </c>
       <c r="O51">
         <f t="shared" si="1"/>
-        <v>-5.7210916898170883</v>
+        <v>-0.57210916898170872</v>
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
@@ -3244,7 +3257,7 @@
       </c>
       <c r="O52">
         <f t="shared" si="1"/>
-        <v>-5.3865828855703448</v>
+        <v>-0.53865828855703457</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
@@ -3293,7 +3306,7 @@
       </c>
       <c r="O53">
         <f t="shared" si="1"/>
-        <v>-5.0518262970241583</v>
+        <v>-0.50518262970241579</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
@@ -3342,7 +3355,7 @@
       </c>
       <c r="O54">
         <f t="shared" si="1"/>
-        <v>-4.7168219241785305</v>
+        <v>-0.47168219241785303</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
@@ -3391,7 +3404,7 @@
       </c>
       <c r="O55">
         <f t="shared" si="1"/>
-        <v>-4.3813219827340184</v>
+        <v>-0.43813219827340183</v>
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
@@ -3440,7 +3453,7 @@
       </c>
       <c r="O56">
         <f t="shared" si="1"/>
-        <v>-4.045574256990065</v>
+        <v>-0.40455742569900643</v>
       </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
@@ -3489,7 +3502,7 @@
       </c>
       <c r="O57">
         <f t="shared" si="1"/>
-        <v>-3.7093309626472268</v>
+        <v>-0.37093309626472265</v>
       </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
@@ -3538,7 +3551,7 @@
       </c>
       <c r="O58">
         <f t="shared" si="1"/>
-        <v>-3.3730876683043882</v>
+        <v>-0.33730876683043881</v>
       </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
@@ -3587,7 +3600,7 @@
       </c>
       <c r="O59">
         <f t="shared" si="1"/>
-        <v>-3.0363488053626662</v>
+        <v>-0.30363488053626658</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
@@ -3636,7 +3649,7 @@
       </c>
       <c r="O60">
         <f t="shared" si="1"/>
-        <v>-2.6996099424209441</v>
+        <v>-0.26996099424209435</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
@@ -3685,7 +3698,7 @@
       </c>
       <c r="O61">
         <f t="shared" si="1"/>
-        <v>-2.3626232951797799</v>
+        <v>-0.23626232951797796</v>
       </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
@@ -3734,7 +3747,7 @@
       </c>
       <c r="O62">
         <f t="shared" si="1"/>
-        <v>-2.0253888636391735</v>
+        <v>-0.20253888636391737</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
@@ -3783,7 +3796,7 @@
       </c>
       <c r="O63">
         <f t="shared" si="1"/>
-        <v>-1.6879066477991256</v>
+        <v>-0.16879066477991256</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
@@ -3832,7 +3845,7 @@
       </c>
       <c r="O64">
         <f t="shared" si="1"/>
-        <v>-1.3504244319590772</v>
+        <v>-0.13504244319590772</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
@@ -3881,7 +3894,7 @@
       </c>
       <c r="O65">
         <f t="shared" si="1"/>
-        <v>-1.0129422161190289</v>
+        <v>-0.10129422161190287</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
@@ -3930,7 +3943,7 @@
       </c>
       <c r="O66">
         <f t="shared" si="1"/>
-        <v>-0.67521221597953862</v>
+        <v>-6.7521221597953859E-2</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
@@ -3979,7 +3992,7 @@
       </c>
       <c r="O67">
         <f t="shared" si="1"/>
-        <v>-0.33773000013949028</v>
+        <v>-3.3773000013949027E-2</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
@@ -4077,7 +4090,7 @@
       </c>
       <c r="O69">
         <f t="shared" si="1"/>
-        <v>0.33773000013949028</v>
+        <v>3.3773000013949027E-2</v>
       </c>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
@@ -4126,7 +4139,7 @@
       </c>
       <c r="O70">
         <f t="shared" si="1"/>
-        <v>0.67521221597953862</v>
+        <v>6.7521221597953859E-2</v>
       </c>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.25">
@@ -4175,7 +4188,7 @@
       </c>
       <c r="O71">
         <f t="shared" si="1"/>
-        <v>1.0129422161190289</v>
+        <v>0.10129422161190287</v>
       </c>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.25">
@@ -4224,7 +4237,7 @@
       </c>
       <c r="O72">
         <f t="shared" si="1"/>
-        <v>1.3504244319590772</v>
+        <v>0.13504244319590772</v>
       </c>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.25">
@@ -4272,8 +4285,8 @@
         <v>11345.466125000001</v>
       </c>
       <c r="O73">
-        <f t="shared" ref="O73:O128" si="3">I73*N73*0.18*0.121333</f>
-        <v>1.6876588634996836</v>
+        <f t="shared" ref="O73:O128" si="3">I73*N73*0.018*0.121333</f>
+        <v>0.16876588634996834</v>
       </c>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.25">
@@ -4322,7 +4335,7 @@
       </c>
       <c r="O74">
         <f t="shared" si="3"/>
-        <v>2.0248932950402896</v>
+        <v>0.20248932950402895</v>
       </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.25">
@@ -4371,7 +4384,7 @@
       </c>
       <c r="O75">
         <f t="shared" si="3"/>
-        <v>2.3618799422814538</v>
+        <v>0.23618799422814538</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.25">
@@ -4420,7 +4433,7 @@
       </c>
       <c r="O76">
         <f t="shared" si="3"/>
-        <v>2.698866589522618</v>
+        <v>0.26988665895226177</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.25">
@@ -4469,7 +4482,7 @@
       </c>
       <c r="O77">
         <f t="shared" si="3"/>
-        <v>3.0356054524643405</v>
+        <v>0.303560545246434</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.25">
@@ -4518,7 +4531,7 @@
       </c>
       <c r="O78">
         <f t="shared" si="3"/>
-        <v>3.3718487468071783</v>
+        <v>0.33718487468071784</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.25">
@@ -4567,7 +4580,7 @@
       </c>
       <c r="O79">
         <f t="shared" si="3"/>
-        <v>3.7080920411500164</v>
+        <v>0.37080920411500162</v>
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.25">
@@ -4616,7 +4629,7 @@
       </c>
       <c r="O80">
         <f t="shared" si="3"/>
-        <v>4.0438397668939716</v>
+        <v>0.40438397668939707</v>
       </c>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.25">
@@ -4665,7 +4678,7 @@
       </c>
       <c r="O81">
         <f t="shared" si="3"/>
-        <v>4.379339708338482</v>
+        <v>0.43793397083384816</v>
       </c>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
@@ -4714,7 +4727,7 @@
       </c>
       <c r="O82">
         <f t="shared" si="3"/>
-        <v>4.7145918654835519</v>
+        <v>0.47145918654835522</v>
       </c>
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.25">
@@ -4763,7 +4776,7 @@
       </c>
       <c r="O83">
         <f t="shared" si="3"/>
-        <v>5.0493484540297384</v>
+        <v>0.50493484540297373</v>
       </c>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.25">
@@ -4812,7 +4825,7 @@
       </c>
       <c r="O84">
         <f t="shared" si="3"/>
-        <v>5.3838572582764828</v>
+        <v>0.53838572582764821</v>
       </c>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.25">
@@ -4861,7 +4874,7 @@
       </c>
       <c r="O85">
         <f t="shared" si="3"/>
-        <v>5.7178704939243419</v>
+        <v>0.57178704939243408</v>
       </c>
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.25">
@@ -4910,7 +4923,7 @@
       </c>
       <c r="O86">
         <f t="shared" si="3"/>
-        <v>6.0513881609733176</v>
+        <v>0.60513881609733178</v>
       </c>
     </row>
     <row r="87" spans="1:15" x14ac:dyDescent="0.25">
@@ -4959,7 +4972,7 @@
       </c>
       <c r="O87">
         <f t="shared" si="3"/>
-        <v>6.3844102594234098</v>
+        <v>0.63844102594234098</v>
       </c>
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.25">
@@ -5008,7 +5021,7 @@
       </c>
       <c r="O88">
         <f t="shared" si="3"/>
-        <v>6.7171845735740598</v>
+        <v>0.67171845735740587</v>
       </c>
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.25">
@@ -5057,7 +5070,7 @@
       </c>
       <c r="O89">
         <f t="shared" si="3"/>
-        <v>7.0492155348263834</v>
+        <v>0.70492155348263819</v>
       </c>
     </row>
     <row r="90" spans="1:15" x14ac:dyDescent="0.25">
@@ -5106,7 +5119,7 @@
       </c>
       <c r="O90">
         <f t="shared" si="3"/>
-        <v>7.3807509274798226</v>
+        <v>0.73807509274798222</v>
       </c>
     </row>
     <row r="91" spans="1:15" x14ac:dyDescent="0.25">
@@ -5155,7 +5168,7 @@
       </c>
       <c r="O91">
         <f t="shared" si="3"/>
-        <v>7.7115429672349363</v>
+        <v>0.77115429672349356</v>
       </c>
     </row>
     <row r="92" spans="1:15" x14ac:dyDescent="0.25">
@@ -5204,7 +5217,7 @@
       </c>
       <c r="O92">
         <f t="shared" si="3"/>
-        <v>8.0418394383911647</v>
+        <v>0.8041839438391164</v>
       </c>
     </row>
     <row r="93" spans="1:15" x14ac:dyDescent="0.25">
@@ -5253,7 +5266,7 @@
       </c>
       <c r="O93">
         <f t="shared" si="3"/>
-        <v>8.3716403409485078</v>
+        <v>0.83716403409485085</v>
       </c>
     </row>
     <row r="94" spans="1:15" x14ac:dyDescent="0.25">
@@ -5302,7 +5315,7 @@
       </c>
       <c r="O94">
         <f t="shared" si="3"/>
-        <v>8.700697890607529</v>
+        <v>0.87006978906075294</v>
       </c>
     </row>
     <row r="95" spans="1:15" x14ac:dyDescent="0.25">
@@ -5351,7 +5364,7 @@
       </c>
       <c r="O95">
         <f t="shared" si="3"/>
-        <v>9.029259871667664</v>
+        <v>0.90292598716676642</v>
       </c>
     </row>
     <row r="96" spans="1:15" x14ac:dyDescent="0.25">
@@ -5400,7 +5413,7 @@
       </c>
       <c r="O96">
         <f t="shared" si="3"/>
-        <v>9.3568307155300303</v>
+        <v>0.93568307155300301</v>
       </c>
     </row>
     <row r="97" spans="1:15" x14ac:dyDescent="0.25">
@@ -5449,7 +5462,7 @@
       </c>
       <c r="O97">
         <f t="shared" si="3"/>
-        <v>9.6839059907935141</v>
+        <v>0.96839059907935143</v>
       </c>
     </row>
     <row r="98" spans="1:15" x14ac:dyDescent="0.25">
@@ -5498,7 +5511,7 @@
       </c>
       <c r="O98">
         <f t="shared" si="3"/>
-        <v>10.009990128859231</v>
+        <v>1.000999012885923</v>
       </c>
     </row>
     <row r="99" spans="1:15" x14ac:dyDescent="0.25">
@@ -5547,7 +5560,7 @@
       </c>
       <c r="O99">
         <f t="shared" si="3"/>
-        <v>10.335578698326058</v>
+        <v>1.033557869832606</v>
       </c>
     </row>
     <row r="100" spans="1:15" x14ac:dyDescent="0.25">
@@ -5596,7 +5609,7 @@
       </c>
       <c r="O100">
         <f t="shared" si="3"/>
-        <v>10.660176130595122</v>
+        <v>1.066017613059512</v>
       </c>
     </row>
     <row r="101" spans="1:15" x14ac:dyDescent="0.25">
@@ -5645,7 +5658,7 @@
       </c>
       <c r="O101">
         <f t="shared" si="3"/>
-        <v>10.984030209965859</v>
+        <v>1.0984030209965858</v>
       </c>
     </row>
     <row r="102" spans="1:15" x14ac:dyDescent="0.25">
@@ -5694,7 +5707,7 @@
       </c>
       <c r="O102">
         <f t="shared" si="3"/>
-        <v>11.306893152138827</v>
+        <v>1.1306893152138826</v>
       </c>
     </row>
     <row r="103" spans="1:15" x14ac:dyDescent="0.25">
@@ -5743,7 +5756,7 @@
       </c>
       <c r="O103">
         <f t="shared" si="3"/>
-        <v>11.629012741413469</v>
+        <v>1.1629012741413469</v>
       </c>
     </row>
     <row r="104" spans="1:15" x14ac:dyDescent="0.25">
@@ -5792,7 +5805,7 @@
       </c>
       <c r="O104">
         <f t="shared" si="3"/>
-        <v>11.950388977789784</v>
+        <v>1.1950388977789785</v>
       </c>
     </row>
     <row r="105" spans="1:15" x14ac:dyDescent="0.25">
@@ -5841,7 +5854,7 @@
       </c>
       <c r="O105">
         <f t="shared" si="3"/>
-        <v>12.270774076968333</v>
+        <v>1.2270774076968334</v>
       </c>
     </row>
     <row r="106" spans="1:15" x14ac:dyDescent="0.25">
@@ -5890,7 +5903,7 @@
       </c>
       <c r="O106">
         <f t="shared" si="3"/>
-        <v>12.589920254649671</v>
+        <v>1.2589920254649671</v>
       </c>
     </row>
     <row r="107" spans="1:15" x14ac:dyDescent="0.25">
@@ -5939,7 +5952,7 @@
       </c>
       <c r="O107">
         <f t="shared" si="3"/>
-        <v>12.908323079432686</v>
+        <v>1.2908323079432684</v>
       </c>
     </row>
     <row r="108" spans="1:15" x14ac:dyDescent="0.25">
@@ -5988,7 +6001,7 @@
       </c>
       <c r="O108">
         <f t="shared" si="3"/>
-        <v>13.225734767017927</v>
+        <v>1.3225734767017927</v>
       </c>
     </row>
     <row r="109" spans="1:15" x14ac:dyDescent="0.25">
@@ -6037,7 +6050,7 @@
       </c>
       <c r="O109">
         <f t="shared" si="3"/>
-        <v>13.542155317405403</v>
+        <v>1.3542155317405402</v>
       </c>
     </row>
     <row r="110" spans="1:15" x14ac:dyDescent="0.25">
@@ -6086,7 +6099,7 @@
       </c>
       <c r="O110">
         <f t="shared" si="3"/>
-        <v>13.857584730595109</v>
+        <v>1.3857584730595107</v>
       </c>
     </row>
     <row r="111" spans="1:15" x14ac:dyDescent="0.25">
@@ -6135,7 +6148,7 @@
       </c>
       <c r="O111">
         <f t="shared" si="3"/>
-        <v>14.171775222287609</v>
+        <v>1.4171775222287608</v>
       </c>
     </row>
     <row r="112" spans="1:15" x14ac:dyDescent="0.25">
@@ -6184,7 +6197,7 @@
       </c>
       <c r="O112">
         <f t="shared" si="3"/>
-        <v>14.484974576782335</v>
+        <v>1.4484974576782335</v>
       </c>
     </row>
     <row r="113" spans="1:15" x14ac:dyDescent="0.25">
@@ -6233,7 +6246,7 @@
       </c>
       <c r="O113">
         <f t="shared" si="3"/>
-        <v>14.796935009779853</v>
+        <v>1.4796935009779855</v>
       </c>
     </row>
     <row r="114" spans="1:15" x14ac:dyDescent="0.25">
@@ -6282,7 +6295,7 @@
       </c>
       <c r="O114">
         <f t="shared" si="3"/>
-        <v>15.107904305579607</v>
+        <v>1.5107904305579607</v>
       </c>
     </row>
     <row r="115" spans="1:15" x14ac:dyDescent="0.25">
@@ -6331,7 +6344,7 @@
       </c>
       <c r="O115">
         <f t="shared" si="3"/>
-        <v>15.417634679882147</v>
+        <v>1.5417634679882146</v>
       </c>
     </row>
     <row r="116" spans="1:15" x14ac:dyDescent="0.25">
@@ -6380,7 +6393,7 @@
       </c>
       <c r="O116">
         <f t="shared" si="3"/>
-        <v>15.726373916986915</v>
+        <v>1.5726373916986915</v>
       </c>
     </row>
     <row r="117" spans="1:15" x14ac:dyDescent="0.25">
@@ -6429,7 +6442,7 @@
       </c>
       <c r="O117">
         <f t="shared" si="3"/>
-        <v>16.033626448295038</v>
+        <v>1.6033626448295037</v>
       </c>
     </row>
     <row r="118" spans="1:15" x14ac:dyDescent="0.25">
@@ -6478,7 +6491,7 @@
       </c>
       <c r="O118">
         <f t="shared" si="3"/>
-        <v>16.339887842405393</v>
+        <v>1.6339887842405389</v>
       </c>
     </row>
     <row r="119" spans="1:15" x14ac:dyDescent="0.25">
@@ -6527,7 +6540,7 @@
       </c>
       <c r="O119">
         <f t="shared" si="3"/>
-        <v>16.644662530719092</v>
+        <v>1.664466253071909</v>
       </c>
     </row>
     <row r="120" spans="1:15" x14ac:dyDescent="0.25">
@@ -6576,7 +6589,7 @@
       </c>
       <c r="O120">
         <f t="shared" si="3"/>
-        <v>16.948198297535583</v>
+        <v>1.6948198297535582</v>
       </c>
     </row>
     <row r="121" spans="1:15" x14ac:dyDescent="0.25">
@@ -6625,7 +6638,7 @@
       </c>
       <c r="O121">
         <f t="shared" si="3"/>
-        <v>17.250495142854859</v>
+        <v>1.7250495142854863</v>
       </c>
     </row>
     <row r="122" spans="1:15" x14ac:dyDescent="0.25">
@@ -6674,7 +6687,7 @@
       </c>
       <c r="O122">
         <f t="shared" si="3"/>
-        <v>17.551553066676927</v>
+        <v>1.7551553066676928</v>
       </c>
     </row>
     <row r="123" spans="1:15" x14ac:dyDescent="0.25">
@@ -6723,7 +6736,7 @@
       </c>
       <c r="O123">
         <f t="shared" si="3"/>
-        <v>17.851124284702347</v>
+        <v>1.7851124284702347</v>
       </c>
     </row>
     <row r="124" spans="1:15" x14ac:dyDescent="0.25">
@@ -6772,7 +6785,7 @@
       </c>
       <c r="O124">
         <f t="shared" si="3"/>
-        <v>18.149456581230556</v>
+        <v>1.8149456581230556</v>
       </c>
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.25">
@@ -6821,7 +6834,7 @@
       </c>
       <c r="O125">
         <f t="shared" si="3"/>
-        <v>18.44630217196211</v>
+        <v>1.8446302171962108</v>
       </c>
     </row>
     <row r="126" spans="1:15" x14ac:dyDescent="0.25">
@@ -6870,7 +6883,7 @@
       </c>
       <c r="O126">
         <f t="shared" si="3"/>
-        <v>18.741661056897012</v>
+        <v>1.874166105689701</v>
       </c>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.25">
@@ -6919,7 +6932,7 @@
       </c>
       <c r="O127">
         <f t="shared" si="3"/>
-        <v>19.035781020334706</v>
+        <v>1.9035781020334706</v>
       </c>
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.25">
@@ -6968,7 +6981,7 @@
       </c>
       <c r="O128">
         <f t="shared" si="3"/>
-        <v>19.32841427797575</v>
+        <v>1.9328414277975747</v>
       </c>
     </row>
   </sheetData>

</xml_diff>